<commit_message>
Add Hum Nat rev
</commit_message>
<xml_diff>
--- a/data/editorial_en.xlsx
+++ b/data/editorial_en.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="65">
   <si>
     <t xml:space="preserve">what</t>
   </si>
@@ -174,6 +174,9 @@
   </si>
   <si>
     <t xml:space="preserve">\href{https://www.sciencedirect.com/journal/cortex}{Cortex}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">\href{https://link.springer.com/journal/12110}{Human Nature}</t>
   </si>
   <si>
     <t xml:space="preserve">\href{https://www.springer.com/journal/10919/}{Journal of Nonverbal Behavior}</t>
@@ -223,7 +226,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -252,6 +255,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -296,7 +305,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -315,6 +324,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -337,37 +350,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
@@ -506,7 +519,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E1048576"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultColWidth="11.43359375" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.3"/>
@@ -788,18 +801,18 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
-      <c r="B25" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="5" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
+      <c r="B26" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
@@ -817,22 +830,22 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
-      <c r="B28" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
+      <c r="B29" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -846,46 +859,46 @@
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
-      <c r="B31" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
+      <c r="B32" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="2" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="B34" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="D34" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
       <c r="E34" s="2" t="s">
         <v>63</v>
       </c>
@@ -895,7 +908,9 @@
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
+      <c r="E35" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2"/>
@@ -918,12 +933,19 @@
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
     </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E4" r:id="rId1" display="https://evohuman.org/edhb/editorial-board"/>
+    <hyperlink ref="E4" r:id="rId1" display="\href{https://evohuman.org/edhb/editorial-board}{Editorial Board}"/>
     <hyperlink ref="E11" r:id="rId2" display="Theme Issue \textbf{\textit{Voice modulation: from origin and mechanism to social impact}} (\href{https://royalsocietypublishing.org/toc/rstb/2021/376/1840}{\textbf{Part 1}}, \href{https://royalsocietypublishing.org/toc/rstb/2022/377/1841}{\textbf{Part 2}})"/>
     <hyperlink ref="E19" r:id="rId3" display="\href{https://nyaspubs.onlinelibrary.wiley.com/journal/17496632}{Annals of the New York Academy of Sciences}"/>
+    <hyperlink ref="E25" r:id="rId4" display="https://link.springer.com/journal/12110"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>